<commit_message>
Update ETF data and clean old Excel files
</commit_message>
<xml_diff>
--- a/etf_holdings/2026-09-13_00400A_full_holdings.xlsx
+++ b/etf_holdings/2026-09-13_00400A_full_holdings.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:51</t>
+          <t>2026-09-13 21:54:59</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:52</t>
+          <t>2026-09-13 21:55:01</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:54</t>
+          <t>2026-09-13 21:55:02</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:55</t>
+          <t>2026-09-13 21:55:03</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:55</t>
+          <t>2026-09-13 21:55:03</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:55</t>
+          <t>2026-09-13 21:55:03</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:55</t>
+          <t>2026-09-13 21:55:03</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-09-13 21:51:55</t>
+          <t>2026-09-13 21:55:03</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">

</xml_diff>